<commit_message>
Update job search data from run 6
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -28078,7 +28078,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28135,11 +28135,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-16T21:02:36.618455</t>
+          <t>2026-06-16T21:42:28.671494</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -28155,12 +28155,45 @@
         <v>400</v>
       </c>
       <c r="H2" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-16T21:02:36.618455</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>400</v>
+      </c>
+      <c r="H3" t="n">
+        <v>400</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
@@ -28597,7 +28630,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>

</xml_diff>